<commit_message>
Tone the 2027 manager targets down to 65% of the plan's growth
Each month's target is now the same month of 2026 plus 65% of what our
plan adds (a café the plan grows 20% gets +13%, one at 10% gets +6.5%), so
quarters and years keep exactly 65% of the plan's growth. The nine cafés'
targets go from $31.30M (+12.6%) to $30.07M (+8.2%), still $1.36M over
today's run-rate and $1.25M over the budget; with La Jolla Cove, whose
remodeled Oct-Dec 2027 stays at the budget's $125K a month, $30.96M.
Every café stays above its run-rate; La Jolla Juicery ends $19K under its
budget.

The deck explains the rule (summary, how the targets are built,
definitions, targets overview), the workbook notes say so, and a check
ties the nine's growth to 65% of the plan's. On the quarterly slide the
2027 bars drop their value labels, which the table beside the chart gives.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C2c9kVN8V8siaKQgSRcGwk
</commit_message>
<xml_diff>
--- a/outputs/Parakeet_2027_Manager_Targets.xlsx
+++ b/outputs/Parakeet_2027_Manager_Targets.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Parakeet Café · 2027 sales targets by store</t>
   </si>
   <si>
-    <t xml:space="preserve">Net sales targets per month (our plan; La Jolla Cove switches to the budget's remodeled rate from its Oct 1, 2027 reopening). Blue = values from the analysis; black = formulas.</t>
+    <t xml:space="preserve">Net sales targets per month (each month of 2026 plus 65% of the growth in our plan; La Jolla Cove switches to the budget's remodeled rate from its Oct 1, 2027 reopening). Blue = values from the analysis; black = formulas.</t>
   </si>
   <si>
     <t xml:space="preserve">Store</t>
@@ -209,7 +209,7 @@
     <t xml:space="preserve">Reference: 2026 finish and 2027 under each view</t>
   </si>
   <si>
-    <t xml:space="preserve">Sources: Toast POS net sales through Oct 14, 2026; investor budget workbook (2027_Sales_budget_Investors.xlsx); run-rate = last 45 days seasonally adjusted; target = our plan.</t>
+    <t xml:space="preserve">Sources: Toast POS net sales through Oct 14, 2026; investor budget workbook (2027_Sales_budget_Investors.xlsx); run-rate = last 45 days seasonally adjusted; target = each month of 2026 plus 65% of the growth in our plan.</t>
   </si>
   <si>
     <t xml:space="preserve">2025 actual (Toast)</t>
@@ -789,67 +789,67 @@
         <v>22</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>240335.44</v>
+        <v>222665.72</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>232184.11</v>
+        <v>215270.61</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>257387.11</v>
+        <v>237349.22</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>248190.77</v>
+        <v>230307.13</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>272444.59</v>
+        <v>255311.3</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>263775.07</v>
+        <v>248397</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>269201.25</v>
+        <v>255876.37</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>281751.13</v>
+        <v>267229.53</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>256443.1</v>
+        <v>241289.02</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>265311.55</v>
+        <v>259364.53</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>266803.98</v>
+        <v>255086.19</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>265578.91</v>
+        <v>251729.39</v>
       </c>
       <c r="N5" s="7" t="n">
         <f aca="false">SUM(B5:D5)</f>
-        <v>729906.66</v>
+        <v>675285.55</v>
       </c>
       <c r="O5" s="7" t="n">
         <f aca="false">SUM(E5:G5)</f>
-        <v>784410.43</v>
+        <v>734015.43</v>
       </c>
       <c r="P5" s="7" t="n">
         <f aca="false">SUM(H5:J5)</f>
-        <v>807395.48</v>
+        <v>764394.92</v>
       </c>
       <c r="Q5" s="7" t="n">
         <f aca="false">SUM(K5:M5)</f>
-        <v>797694.44</v>
+        <v>766180.11</v>
       </c>
       <c r="R5" s="7" t="n">
         <f aca="false">SUM(B5:M5)</f>
-        <v>3119407.01</v>
+        <v>2939876.01</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>2606461.36</v>
       </c>
       <c r="T5" s="8" t="n">
         <f aca="false">IF(S5=0,"",R5/S5-1)</f>
-        <v>0.196797718881204</v>
+        <v>0.127918508640389</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -857,67 +857,67 @@
         <v>23</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>227289.23</v>
+        <v>216903.56</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>203905.78</v>
+        <v>197302.72</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>222438.88</v>
+        <v>213363.55</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>214066.03</v>
+        <v>204892.53</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>230110.53</v>
+        <v>220729.95</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>204562.27</v>
+        <v>196692.96</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>205433.25</v>
+        <v>195722.16</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>216074.01</v>
+        <v>207693.16</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>215120.82</v>
+        <v>204606.16</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>238271.16</v>
+        <v>225681.87</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>237928.07</v>
+        <v>226121.26</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>226464.41</v>
+        <v>213400.77</v>
       </c>
       <c r="N6" s="7" t="n">
         <f aca="false">SUM(B6:D6)</f>
-        <v>653633.89</v>
+        <v>627569.83</v>
       </c>
       <c r="O6" s="7" t="n">
         <f aca="false">SUM(E6:G6)</f>
-        <v>648738.83</v>
+        <v>622315.44</v>
       </c>
       <c r="P6" s="7" t="n">
         <f aca="false">SUM(H6:J6)</f>
-        <v>636628.08</v>
+        <v>608021.48</v>
       </c>
       <c r="Q6" s="7" t="n">
         <f aca="false">SUM(K6:M6)</f>
-        <v>702663.64</v>
+        <v>665203.9</v>
       </c>
       <c r="R6" s="7" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>2641664.44</v>
+        <v>2523110.65</v>
       </c>
       <c r="S6" s="6" t="n">
         <v>2302939.27</v>
       </c>
       <c r="T6" s="8" t="n">
         <f aca="false">IF(S6=0,"",R6/S6-1)</f>
-        <v>0.147083848198915</v>
+        <v>0.0956045097967346</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -925,67 +925,67 @@
         <v>24</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>347155.87</v>
+        <v>330798.67</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>303859.01</v>
+        <v>290557.85</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>350055.72</v>
+        <v>339834.76</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>355295.68</v>
+        <v>341465.42</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>381551.8</v>
+        <v>367770.12</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>347223.39</v>
+        <v>331617.91</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>370112.79</v>
+        <v>349316.1</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>362058.09</v>
+        <v>349628.43</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>325338.38</v>
+        <v>313971.35</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>343803.24</v>
+        <v>326866.99</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>356440.28</v>
+        <v>341564.38</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>390772.6</v>
+        <v>371766.59</v>
       </c>
       <c r="N7" s="7" t="n">
         <f aca="false">SUM(B7:D7)</f>
-        <v>1001070.6</v>
+        <v>961191.28</v>
       </c>
       <c r="O7" s="7" t="n">
         <f aca="false">SUM(E7:G7)</f>
-        <v>1084070.87</v>
+        <v>1040853.45</v>
       </c>
       <c r="P7" s="7" t="n">
         <f aca="false">SUM(H7:J7)</f>
-        <v>1057509.26</v>
+        <v>1012915.88</v>
       </c>
       <c r="Q7" s="7" t="n">
         <f aca="false">SUM(K7:M7)</f>
-        <v>1091016.12</v>
+        <v>1040197.96</v>
       </c>
       <c r="R7" s="7" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>4233666.85</v>
+        <v>4055158.57</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>3723643.18</v>
       </c>
       <c r="T7" s="8" t="n">
         <f aca="false">IF(S7=0,"",R7/S7-1)</f>
-        <v>0.136968996583609</v>
+        <v>0.0890298489878398</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -993,67 +993,67 @@
         <v>25</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>312399.46</v>
+        <v>304631.98</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>281595.6</v>
+        <v>275671.13</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>362333.45</v>
+        <v>364481.8</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>356921.7</v>
+        <v>347969.67</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>376891.75</v>
+        <v>373536.14</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>378275.27</v>
+        <v>366821.39</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>516508.85</v>
+        <v>499555.29</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>427274.35</v>
+        <v>418224.45</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>310518.86</v>
+        <v>301447.17</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>327674.08</v>
+        <v>312304.44</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>306577.59</v>
+        <v>296489.07</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>350719.75</v>
+        <v>334478.77</v>
       </c>
       <c r="N8" s="7" t="n">
         <f aca="false">SUM(B8:D8)</f>
-        <v>956328.51</v>
+        <v>944784.91</v>
       </c>
       <c r="O8" s="7" t="n">
         <f aca="false">SUM(E8:G8)</f>
-        <v>1112088.72</v>
+        <v>1088327.2</v>
       </c>
       <c r="P8" s="7" t="n">
         <f aca="false">SUM(H8:J8)</f>
-        <v>1254302.06</v>
+        <v>1219226.91</v>
       </c>
       <c r="Q8" s="7" t="n">
         <f aca="false">SUM(K8:M8)</f>
-        <v>984971.42</v>
+        <v>943272.28</v>
       </c>
       <c r="R8" s="7" t="n">
         <f aca="false">SUM(B8:M8)</f>
-        <v>4307690.71</v>
+        <v>4195611.3</v>
       </c>
       <c r="S8" s="6" t="n">
         <v>3987463.81</v>
       </c>
       <c r="T8" s="8" t="n">
         <f aca="false">IF(S8=0,"",R8/S8-1)</f>
-        <v>0.0803084153884772</v>
+        <v>0.0522004712564399</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1061,67 +1061,67 @@
         <v>26</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>430949.59</v>
+        <v>415428.35</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>383310.31</v>
+        <v>371270.04</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>438484.65</v>
+        <v>426811.77</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>416409.53</v>
+        <v>402678.17</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>454594.01</v>
+        <v>437964.65</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>421443.45</v>
+        <v>406798.74</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>444464.45</v>
+        <v>426643.14</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>462061.08</v>
+        <v>452114.45</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>403897.6</v>
+        <v>390804.77</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>425684.45</v>
+        <v>412075.95</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>416009.75</v>
+        <v>402337.19</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>453974.83</v>
+        <v>436438.26</v>
       </c>
       <c r="N9" s="7" t="n">
         <f aca="false">SUM(B9:D9)</f>
-        <v>1252744.55</v>
+        <v>1213510.16</v>
       </c>
       <c r="O9" s="7" t="n">
         <f aca="false">SUM(E9:G9)</f>
-        <v>1292446.99</v>
+        <v>1247441.56</v>
       </c>
       <c r="P9" s="7" t="n">
         <f aca="false">SUM(H9:J9)</f>
-        <v>1310423.13</v>
+        <v>1269562.36</v>
       </c>
       <c r="Q9" s="7" t="n">
         <f aca="false">SUM(K9:M9)</f>
-        <v>1295669.03</v>
+        <v>1250851.4</v>
       </c>
       <c r="R9" s="7" t="n">
         <f aca="false">SUM(B9:M9)</f>
-        <v>5151283.7</v>
+        <v>4981365.48</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>4665803.06</v>
       </c>
       <c r="T9" s="8" t="n">
         <f aca="false">IF(S9=0,"",R9/S9-1)</f>
-        <v>0.104050821210615</v>
+        <v>0.0676330346442011</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1129,67 +1129,67 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>257347.15</v>
+        <v>249935.35</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>234138.23</v>
+        <v>228766.86</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>265056.56</v>
+        <v>260996.01</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>262039.19</v>
+        <v>252237.93</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>279695.99</v>
+        <v>273929.29</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>254919.15</v>
+        <v>247214.98</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>278642.95</v>
+        <v>269489.88</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>278428.66</v>
+        <v>274315.81</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>244515.81</v>
+        <v>238484.98</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>257847.21</v>
+        <v>252570.07</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>250121.21</v>
+        <v>244479.98</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>264806</v>
+        <v>256922.52</v>
       </c>
       <c r="N10" s="7" t="n">
         <f aca="false">SUM(B10:D10)</f>
-        <v>756541.94</v>
+        <v>739698.22</v>
       </c>
       <c r="O10" s="7" t="n">
         <f aca="false">SUM(E10:G10)</f>
-        <v>796654.33</v>
+        <v>773382.2</v>
       </c>
       <c r="P10" s="7" t="n">
         <f aca="false">SUM(H10:J10)</f>
-        <v>801587.42</v>
+        <v>782290.67</v>
       </c>
       <c r="Q10" s="7" t="n">
         <f aca="false">SUM(K10:M10)</f>
-        <v>772774.42</v>
+        <v>753972.57</v>
       </c>
       <c r="R10" s="7" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>3127558.11</v>
+        <v>3049343.66</v>
       </c>
       <c r="S10" s="6" t="n">
         <v>2904088.3</v>
       </c>
       <c r="T10" s="8" t="n">
         <f aca="false">IF(S10=0,"",R10/S10-1)</f>
-        <v>0.0769500741420295</v>
+        <v>0.0500175425106737</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1197,67 +1197,67 @@
         <v>28</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>70024.33</v>
+        <v>68962.29</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>65363.47</v>
+        <v>64298.16</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>80282.84</v>
+        <v>80750.82</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>78691.41</v>
+        <v>76408.93</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>81914.6</v>
+        <v>81062.97</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>80680.83</v>
+        <v>79234.8</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>95117.93</v>
+        <v>93765.52</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>92412.44</v>
+        <v>92719.44</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>75560.91</v>
+        <v>73936.93</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>74362.39</v>
+        <v>72624.46</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>67804.32</v>
+        <v>66319.24</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>69510.22</v>
+        <v>67419.34</v>
       </c>
       <c r="N11" s="7" t="n">
         <f aca="false">SUM(B11:D11)</f>
-        <v>215670.64</v>
+        <v>214011.27</v>
       </c>
       <c r="O11" s="7" t="n">
         <f aca="false">SUM(E11:G11)</f>
-        <v>241286.84</v>
+        <v>236706.7</v>
       </c>
       <c r="P11" s="7" t="n">
         <f aca="false">SUM(H11:J11)</f>
-        <v>263091.28</v>
+        <v>260421.89</v>
       </c>
       <c r="Q11" s="7" t="n">
         <f aca="false">SUM(K11:M11)</f>
-        <v>211676.93</v>
+        <v>206363.04</v>
       </c>
       <c r="R11" s="7" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>931725.69</v>
+        <v>917502.9</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>891089.16</v>
       </c>
       <c r="T11" s="8" t="n">
         <f aca="false">IF(S11=0,"",R11/S11-1)</f>
-        <v>0.0456032143854157</v>
+        <v>0.0296420843005205</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1265,67 +1265,67 @@
         <v>29</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>296914.31</v>
+        <v>272028.46</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>286294.25</v>
+        <v>262868.2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>338579.82</v>
+        <v>321610.48</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>342033.7</v>
+        <v>321350.71</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>347090.01</v>
+        <v>327929.65</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>332147.99</v>
+        <v>311502.27</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>367354.16</v>
+        <v>345099.66</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>368327.3</v>
+        <v>352910.33</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>307233.84</v>
+        <v>290355.8</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>316289.17</v>
+        <v>299061.64</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>306667.72</v>
+        <v>289356.18</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>319163.66</v>
+        <v>296212.08</v>
       </c>
       <c r="N12" s="7" t="n">
         <f aca="false">SUM(B12:D12)</f>
-        <v>921788.38</v>
+        <v>856507.14</v>
       </c>
       <c r="O12" s="7" t="n">
         <f aca="false">SUM(E12:G12)</f>
-        <v>1021271.7</v>
+        <v>960782.63</v>
       </c>
       <c r="P12" s="7" t="n">
         <f aca="false">SUM(H12:J12)</f>
-        <v>1042915.3</v>
+        <v>988365.79</v>
       </c>
       <c r="Q12" s="7" t="n">
         <f aca="false">SUM(K12:M12)</f>
-        <v>942120.55</v>
+        <v>884629.9</v>
       </c>
       <c r="R12" s="7" t="n">
         <f aca="false">SUM(B12:M12)</f>
-        <v>3928095.93</v>
+        <v>3690285.46</v>
       </c>
       <c r="S12" s="6" t="n">
         <v>3248637.47</v>
       </c>
       <c r="T12" s="8" t="n">
         <f aca="false">IF(S12=0,"",R12/S12-1)</f>
-        <v>0.209151826350141</v>
+        <v>0.135948684357199</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1333,67 +1333,67 @@
         <v>30</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>327146.38</v>
+        <v>310339.79</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>271492.7</v>
+        <v>261447.34</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>316609.81</v>
+        <v>310773.11</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>307133.63</v>
+        <v>296667.43</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>349631.07</v>
+        <v>339151.24</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>326325.44</v>
+        <v>316744.84</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>363061.05</v>
+        <v>349578</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>359674.68</v>
+        <v>352910.43</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>296046.26</v>
+        <v>285576.59</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>317470.65</v>
+        <v>300807.14</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>297737.89</v>
+        <v>287803.85</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>322139.38</v>
+        <v>306150.86</v>
       </c>
       <c r="N13" s="7" t="n">
         <f aca="false">SUM(B13:D13)</f>
-        <v>915248.89</v>
+        <v>882560.24</v>
       </c>
       <c r="O13" s="7" t="n">
         <f aca="false">SUM(E13:G13)</f>
-        <v>983090.14</v>
+        <v>952563.51</v>
       </c>
       <c r="P13" s="7" t="n">
         <f aca="false">SUM(H13:J13)</f>
-        <v>1018781.99</v>
+        <v>988065.02</v>
       </c>
       <c r="Q13" s="7" t="n">
         <f aca="false">SUM(K13:M13)</f>
-        <v>937347.92</v>
+        <v>894761.85</v>
       </c>
       <c r="R13" s="7" t="n">
         <f aca="false">SUM(B13:M13)</f>
-        <v>3854468.94</v>
+        <v>3717950.62</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>3464416.6</v>
       </c>
       <c r="T13" s="8" t="n">
         <f aca="false">IF(S13=0,"",R13/S13-1)</f>
-        <v>0.112588174297514</v>
+        <v>0.0731823130047349</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1402,71 +1402,71 @@
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">SUM(B5:B13)</f>
-        <v>2509561.76</v>
+        <v>2391694.17</v>
       </c>
       <c r="C14" s="10" t="n">
         <f aca="false">SUM(C5:C13)</f>
-        <v>2262143.46</v>
+        <v>2167452.91</v>
       </c>
       <c r="D14" s="10" t="n">
         <f aca="false">SUM(D5:D13)</f>
-        <v>2631228.84</v>
+        <v>2555971.52</v>
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">SUM(E5:E13)</f>
-        <v>2580781.64</v>
+        <v>2473977.92</v>
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">SUM(F5:F13)</f>
-        <v>2773924.35</v>
+        <v>2677385.31</v>
       </c>
       <c r="G14" s="10" t="n">
         <f aca="false">SUM(G5:G13)</f>
-        <v>2609352.86</v>
+        <v>2505024.89</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">SUM(H5:H13)</f>
-        <v>2909896.68</v>
+        <v>2785046.12</v>
       </c>
       <c r="I14" s="10" t="n">
         <f aca="false">SUM(I5:I13)</f>
-        <v>2848061.74</v>
+        <v>2767746.03</v>
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">SUM(J5:J13)</f>
-        <v>2434675.58</v>
+        <v>2340472.77</v>
       </c>
       <c r="K14" s="10" t="n">
         <f aca="false">SUM(K5:K13)</f>
-        <v>2566713.9</v>
+        <v>2461357.09</v>
       </c>
       <c r="L14" s="10" t="n">
         <f aca="false">SUM(L5:L13)</f>
-        <v>2506090.81</v>
+        <v>2409557.34</v>
       </c>
       <c r="M14" s="10" t="n">
         <f aca="false">SUM(M5:M13)</f>
-        <v>2663129.76</v>
+        <v>2534518.58</v>
       </c>
       <c r="N14" s="10" t="n">
         <f aca="false">SUM(N5:N13)</f>
-        <v>7402934.06</v>
+        <v>7115118.6</v>
       </c>
       <c r="O14" s="10" t="n">
         <f aca="false">SUM(O5:O13)</f>
-        <v>7964058.85</v>
+        <v>7656388.12</v>
       </c>
       <c r="P14" s="10" t="n">
         <f aca="false">SUM(P5:P13)</f>
-        <v>8192634</v>
+        <v>7893264.92</v>
       </c>
       <c r="Q14" s="10" t="n">
         <f aca="false">SUM(Q5:Q13)</f>
-        <v>7735934.47</v>
+        <v>7405433.01</v>
       </c>
       <c r="R14" s="10" t="n">
         <f aca="false">SUM(R5:R13)</f>
-        <v>31295561.38</v>
+        <v>30070204.65</v>
       </c>
       <c r="S14" s="10" t="n">
         <f aca="false">SUM(S5:S13)</f>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="T14" s="11" t="n">
         <f aca="false">IF(S14=0,"",R14/S14-1)</f>
-        <v>0.125960670391628</v>
+        <v>0.0818744350170033</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1482,31 +1482,31 @@
         <v>32</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>49132.16</v>
+        <v>48441.74</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>47789.29</v>
+        <v>47416.51</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>57042.34</v>
+        <v>56982.27</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>58246.45</v>
+        <v>57181.59</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>61613.98</v>
+        <v>60086.27</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>59373.16</v>
+        <v>57726</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>69005.96</v>
+        <v>66755.21</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>63974.68</v>
+        <v>62712.99</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>55593.97</v>
+        <v>54320.07</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>125000</v>
@@ -1519,15 +1519,15 @@
       </c>
       <c r="N15" s="7" t="n">
         <f aca="false">SUM(B15:D15)</f>
-        <v>153963.79</v>
+        <v>152840.52</v>
       </c>
       <c r="O15" s="7" t="n">
         <f aca="false">SUM(E15:G15)</f>
-        <v>179233.59</v>
+        <v>174993.86</v>
       </c>
       <c r="P15" s="7" t="n">
         <f aca="false">SUM(H15:J15)</f>
-        <v>188574.61</v>
+        <v>183788.27</v>
       </c>
       <c r="Q15" s="7" t="n">
         <f aca="false">SUM(K15:M15)</f>
@@ -1535,14 +1535,14 @@
       </c>
       <c r="R15" s="7" t="n">
         <f aca="false">SUM(B15:M15)</f>
-        <v>896771.99</v>
+        <v>886622.65</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>636109.61</v>
       </c>
       <c r="T15" s="8" t="n">
         <f aca="false">IF(S15=0,"",R15/S15-1)</f>
-        <v>0.409775887523536</v>
+        <v>0.393820555548595</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1551,71 +1551,71 @@
       </c>
       <c r="B16" s="10" t="n">
         <f aca="false">B14+B15</f>
-        <v>2558693.92</v>
+        <v>2440135.91</v>
       </c>
       <c r="C16" s="10" t="n">
         <f aca="false">C14+C15</f>
-        <v>2309932.75</v>
+        <v>2214869.42</v>
       </c>
       <c r="D16" s="10" t="n">
         <f aca="false">D14+D15</f>
-        <v>2688271.18</v>
+        <v>2612953.79</v>
       </c>
       <c r="E16" s="10" t="n">
         <f aca="false">E14+E15</f>
-        <v>2639028.09</v>
+        <v>2531159.51</v>
       </c>
       <c r="F16" s="10" t="n">
         <f aca="false">F14+F15</f>
-        <v>2835538.33</v>
+        <v>2737471.58</v>
       </c>
       <c r="G16" s="10" t="n">
         <f aca="false">G14+G15</f>
-        <v>2668726.02</v>
+        <v>2562750.89</v>
       </c>
       <c r="H16" s="10" t="n">
         <f aca="false">H14+H15</f>
-        <v>2978902.64</v>
+        <v>2851801.33</v>
       </c>
       <c r="I16" s="10" t="n">
         <f aca="false">I14+I15</f>
-        <v>2912036.42</v>
+        <v>2830459.02</v>
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">J14+J15</f>
-        <v>2490269.55</v>
+        <v>2394792.84</v>
       </c>
       <c r="K16" s="10" t="n">
         <f aca="false">K14+K15</f>
-        <v>2691713.9</v>
+        <v>2586357.09</v>
       </c>
       <c r="L16" s="10" t="n">
         <f aca="false">L14+L15</f>
-        <v>2631090.81</v>
+        <v>2534557.34</v>
       </c>
       <c r="M16" s="10" t="n">
         <f aca="false">M14+M15</f>
-        <v>2788129.76</v>
+        <v>2659518.58</v>
       </c>
       <c r="N16" s="10" t="n">
         <f aca="false">N14+N15</f>
-        <v>7556897.85</v>
+        <v>7267959.12</v>
       </c>
       <c r="O16" s="10" t="n">
         <f aca="false">O14+O15</f>
-        <v>8143292.44</v>
+        <v>7831381.98</v>
       </c>
       <c r="P16" s="10" t="n">
         <f aca="false">P14+P15</f>
-        <v>8381208.61</v>
+        <v>8077053.19</v>
       </c>
       <c r="Q16" s="10" t="n">
         <f aca="false">Q14+Q15</f>
-        <v>8110934.47</v>
+        <v>7780433.01</v>
       </c>
       <c r="R16" s="10" t="n">
         <f aca="false">R14+R15</f>
-        <v>32192333.37</v>
+        <v>30956827.3</v>
       </c>
       <c r="S16" s="10" t="n">
         <f aca="false">S14+S15</f>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="T16" s="11" t="n">
         <f aca="false">IF(S16=0,"",R16/S16-1)</f>
-        <v>0.132310774083406</v>
+        <v>0.0888539417243652</v>
       </c>
     </row>
   </sheetData>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">'Targets 2027'!R5</f>
-        <v>3119407.01</v>
+        <v>2939876.01</v>
       </c>
       <c r="C5" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A5,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">'Targets 2027'!R6</f>
-        <v>2641664.44</v>
+        <v>2523110.65</v>
       </c>
       <c r="C6" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A6,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">'Targets 2027'!R7</f>
-        <v>4233666.85</v>
+        <v>4055158.57</v>
       </c>
       <c r="C7" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A7,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">'Targets 2027'!R8</f>
-        <v>4307690.71</v>
+        <v>4195611.3</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A8,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">'Targets 2027'!R9</f>
-        <v>5151283.7</v>
+        <v>4981365.48</v>
       </c>
       <c r="C9" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A9,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">'Targets 2027'!R10</f>
-        <v>3127558.11</v>
+        <v>3049343.66</v>
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A10,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">'Targets 2027'!R11</f>
-        <v>931725.69</v>
+        <v>917502.9</v>
       </c>
       <c r="C11" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A11,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">'Targets 2027'!R12</f>
-        <v>3928095.93</v>
+        <v>3690285.46</v>
       </c>
       <c r="C12" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A12,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">'Targets 2027'!R13</f>
-        <v>3854468.94</v>
+        <v>3717950.62</v>
       </c>
       <c r="C13" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A13,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="B14" s="13" t="n">
         <f aca="false">'Targets 2027'!R15</f>
-        <v>896771.99</v>
+        <v>886622.65</v>
       </c>
       <c r="C14" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A14,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="B15" s="10" t="n">
         <f aca="false">SUM(B5:B14)</f>
-        <v>32192333.37</v>
+        <v>30956827.3</v>
       </c>
       <c r="C15" s="10" t="n">
         <f aca="false">SUM(C5:C14)</f>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">'Targets 2027'!B5</f>
-        <v>240335.44</v>
+        <v>222665.72</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="7" t="str">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="C6" s="13" t="n">
         <f aca="false">'Targets 2027'!C5</f>
-        <v>232184.11</v>
+        <v>215270.61</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="7" t="str">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">'Targets 2027'!D5</f>
-        <v>257387.11</v>
+        <v>237349.22</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="7" t="str">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">'Targets 2027'!E5</f>
-        <v>248190.77</v>
+        <v>230307.13</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="7" t="str">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">'Targets 2027'!F5</f>
-        <v>272444.59</v>
+        <v>255311.3</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="7" t="str">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">'Targets 2027'!G5</f>
-        <v>263775.07</v>
+        <v>248397</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="7" t="str">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C11" s="13" t="n">
         <f aca="false">'Targets 2027'!H5</f>
-        <v>269201.25</v>
+        <v>255876.37</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="7" t="str">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="C12" s="13" t="n">
         <f aca="false">'Targets 2027'!I5</f>
-        <v>281751.13</v>
+        <v>267229.53</v>
       </c>
       <c r="D12" s="16"/>
       <c r="E12" s="7" t="str">
@@ -2266,18 +2266,18 @@
       </c>
       <c r="J12" s="13" t="n">
         <f aca="false">C5</f>
-        <v>240335.44</v>
+        <v>222665.72</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>245000</v>
+        <v>227000</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(K12="","",K12-J12)</f>
-        <v>4664.56</v>
+        <v>4334.28</v>
       </c>
       <c r="M12" s="8" t="n">
         <f aca="false">IF(K12="","",K12/J12-1)</f>
-        <v>0.0194085399972639</v>
+        <v>0.0194654120984585</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">'Targets 2027'!J5</f>
-        <v>256443.1</v>
+        <v>241289.02</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="7" t="str">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="C14" s="13" t="n">
         <f aca="false">'Targets 2027'!K5</f>
-        <v>265311.55</v>
+        <v>259364.53</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="7" t="str">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C15" s="13" t="n">
         <f aca="false">'Targets 2027'!L5</f>
-        <v>266803.98</v>
+        <v>255086.19</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="7" t="str">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">'Targets 2027'!M5</f>
-        <v>265578.91</v>
+        <v>251729.39</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="7" t="str">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="C17" s="13" t="n">
         <f aca="false">'Targets 2027'!B6</f>
-        <v>227289.23</v>
+        <v>216903.56</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="7" t="str">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="C18" s="13" t="n">
         <f aca="false">'Targets 2027'!C6</f>
-        <v>203905.78</v>
+        <v>197302.72</v>
       </c>
       <c r="D18" s="16"/>
       <c r="E18" s="7" t="str">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">'Targets 2027'!D6</f>
-        <v>222438.88</v>
+        <v>213363.55</v>
       </c>
       <c r="D19" s="16"/>
       <c r="E19" s="7" t="str">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="C20" s="13" t="n">
         <f aca="false">'Targets 2027'!E6</f>
-        <v>214066.03</v>
+        <v>204892.53</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="7" t="str">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="C21" s="13" t="n">
         <f aca="false">'Targets 2027'!F6</f>
-        <v>230110.53</v>
+        <v>220729.95</v>
       </c>
       <c r="D21" s="16"/>
       <c r="E21" s="7" t="str">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="C22" s="13" t="n">
         <f aca="false">'Targets 2027'!G6</f>
-        <v>204562.27</v>
+        <v>196692.96</v>
       </c>
       <c r="D22" s="16"/>
       <c r="E22" s="7" t="str">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="C23" s="13" t="n">
         <f aca="false">'Targets 2027'!H6</f>
-        <v>205433.25</v>
+        <v>195722.16</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="7" t="str">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="C24" s="13" t="n">
         <f aca="false">'Targets 2027'!I6</f>
-        <v>216074.01</v>
+        <v>207693.16</v>
       </c>
       <c r="D24" s="16"/>
       <c r="E24" s="7" t="str">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C25" s="13" t="n">
         <f aca="false">'Targets 2027'!J6</f>
-        <v>215120.82</v>
+        <v>204606.16</v>
       </c>
       <c r="D25" s="16"/>
       <c r="E25" s="7" t="str">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="C26" s="13" t="n">
         <f aca="false">'Targets 2027'!K6</f>
-        <v>238271.16</v>
+        <v>225681.87</v>
       </c>
       <c r="D26" s="16"/>
       <c r="E26" s="7" t="str">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C27" s="13" t="n">
         <f aca="false">'Targets 2027'!L6</f>
-        <v>237928.07</v>
+        <v>226121.26</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="7" t="str">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="C28" s="13" t="n">
         <f aca="false">'Targets 2027'!M6</f>
-        <v>226464.41</v>
+        <v>213400.77</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="7" t="str">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C29" s="13" t="n">
         <f aca="false">'Targets 2027'!B7</f>
-        <v>347155.87</v>
+        <v>330798.67</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="7" t="str">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="C30" s="13" t="n">
         <f aca="false">'Targets 2027'!C7</f>
-        <v>303859.01</v>
+        <v>290557.85</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="7" t="str">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="C31" s="13" t="n">
         <f aca="false">'Targets 2027'!D7</f>
-        <v>350055.72</v>
+        <v>339834.76</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="7" t="str">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="C32" s="13" t="n">
         <f aca="false">'Targets 2027'!E7</f>
-        <v>355295.68</v>
+        <v>341465.42</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="7" t="str">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C33" s="13" t="n">
         <f aca="false">'Targets 2027'!F7</f>
-        <v>381551.8</v>
+        <v>367770.12</v>
       </c>
       <c r="D33" s="16"/>
       <c r="E33" s="7" t="str">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="C34" s="13" t="n">
         <f aca="false">'Targets 2027'!G7</f>
-        <v>347223.39</v>
+        <v>331617.91</v>
       </c>
       <c r="D34" s="16"/>
       <c r="E34" s="7" t="str">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C35" s="13" t="n">
         <f aca="false">'Targets 2027'!H7</f>
-        <v>370112.79</v>
+        <v>349316.1</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="7" t="str">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C36" s="13" t="n">
         <f aca="false">'Targets 2027'!I7</f>
-        <v>362058.09</v>
+        <v>349628.43</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="7" t="str">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="C37" s="13" t="n">
         <f aca="false">'Targets 2027'!J7</f>
-        <v>325338.38</v>
+        <v>313971.35</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="7" t="str">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C38" s="13" t="n">
         <f aca="false">'Targets 2027'!K7</f>
-        <v>343803.24</v>
+        <v>326866.99</v>
       </c>
       <c r="D38" s="16"/>
       <c r="E38" s="7" t="str">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="C39" s="13" t="n">
         <f aca="false">'Targets 2027'!L7</f>
-        <v>356440.28</v>
+        <v>341564.38</v>
       </c>
       <c r="D39" s="16"/>
       <c r="E39" s="7" t="str">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C40" s="13" t="n">
         <f aca="false">'Targets 2027'!M7</f>
-        <v>390772.6</v>
+        <v>371766.59</v>
       </c>
       <c r="D40" s="16"/>
       <c r="E40" s="7" t="str">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="C41" s="13" t="n">
         <f aca="false">'Targets 2027'!B8</f>
-        <v>312399.46</v>
+        <v>304631.98</v>
       </c>
       <c r="D41" s="16"/>
       <c r="E41" s="7" t="str">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="C42" s="13" t="n">
         <f aca="false">'Targets 2027'!C8</f>
-        <v>281595.6</v>
+        <v>275671.13</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="7" t="str">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="C43" s="13" t="n">
         <f aca="false">'Targets 2027'!D8</f>
-        <v>362333.45</v>
+        <v>364481.8</v>
       </c>
       <c r="D43" s="16"/>
       <c r="E43" s="7" t="str">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="C44" s="13" t="n">
         <f aca="false">'Targets 2027'!E8</f>
-        <v>356921.7</v>
+        <v>347969.67</v>
       </c>
       <c r="D44" s="16"/>
       <c r="E44" s="7" t="str">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="C45" s="13" t="n">
         <f aca="false">'Targets 2027'!F8</f>
-        <v>376891.75</v>
+        <v>373536.14</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="7" t="str">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="C46" s="13" t="n">
         <f aca="false">'Targets 2027'!G8</f>
-        <v>378275.27</v>
+        <v>366821.39</v>
       </c>
       <c r="D46" s="16"/>
       <c r="E46" s="7" t="str">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="C47" s="13" t="n">
         <f aca="false">'Targets 2027'!H8</f>
-        <v>516508.85</v>
+        <v>499555.29</v>
       </c>
       <c r="D47" s="16"/>
       <c r="E47" s="7" t="str">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="C48" s="13" t="n">
         <f aca="false">'Targets 2027'!I8</f>
-        <v>427274.35</v>
+        <v>418224.45</v>
       </c>
       <c r="D48" s="16"/>
       <c r="E48" s="7" t="str">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="C49" s="13" t="n">
         <f aca="false">'Targets 2027'!J8</f>
-        <v>310518.86</v>
+        <v>301447.17</v>
       </c>
       <c r="D49" s="16"/>
       <c r="E49" s="7" t="str">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="C50" s="13" t="n">
         <f aca="false">'Targets 2027'!K8</f>
-        <v>327674.08</v>
+        <v>312304.44</v>
       </c>
       <c r="D50" s="16"/>
       <c r="E50" s="7" t="str">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="C51" s="13" t="n">
         <f aca="false">'Targets 2027'!L8</f>
-        <v>306577.59</v>
+        <v>296489.07</v>
       </c>
       <c r="D51" s="16"/>
       <c r="E51" s="7" t="str">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C52" s="13" t="n">
         <f aca="false">'Targets 2027'!M8</f>
-        <v>350719.75</v>
+        <v>334478.77</v>
       </c>
       <c r="D52" s="16"/>
       <c r="E52" s="7" t="str">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="C53" s="13" t="n">
         <f aca="false">'Targets 2027'!B9</f>
-        <v>430949.59</v>
+        <v>415428.35</v>
       </c>
       <c r="D53" s="16"/>
       <c r="E53" s="7" t="str">
@@ -3150,7 +3150,7 @@
       </c>
       <c r="C54" s="13" t="n">
         <f aca="false">'Targets 2027'!C9</f>
-        <v>383310.31</v>
+        <v>371270.04</v>
       </c>
       <c r="D54" s="16"/>
       <c r="E54" s="7" t="str">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="C55" s="13" t="n">
         <f aca="false">'Targets 2027'!D9</f>
-        <v>438484.65</v>
+        <v>426811.77</v>
       </c>
       <c r="D55" s="16"/>
       <c r="E55" s="7" t="str">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="C56" s="13" t="n">
         <f aca="false">'Targets 2027'!E9</f>
-        <v>416409.53</v>
+        <v>402678.17</v>
       </c>
       <c r="D56" s="16"/>
       <c r="E56" s="7" t="str">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="C57" s="13" t="n">
         <f aca="false">'Targets 2027'!F9</f>
-        <v>454594.01</v>
+        <v>437964.65</v>
       </c>
       <c r="D57" s="16"/>
       <c r="E57" s="7" t="str">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C58" s="13" t="n">
         <f aca="false">'Targets 2027'!G9</f>
-        <v>421443.45</v>
+        <v>406798.74</v>
       </c>
       <c r="D58" s="16"/>
       <c r="E58" s="7" t="str">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="C59" s="13" t="n">
         <f aca="false">'Targets 2027'!H9</f>
-        <v>444464.45</v>
+        <v>426643.14</v>
       </c>
       <c r="D59" s="16"/>
       <c r="E59" s="7" t="str">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C60" s="13" t="n">
         <f aca="false">'Targets 2027'!I9</f>
-        <v>462061.08</v>
+        <v>452114.45</v>
       </c>
       <c r="D60" s="16"/>
       <c r="E60" s="7" t="str">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="C61" s="13" t="n">
         <f aca="false">'Targets 2027'!J9</f>
-        <v>403897.6</v>
+        <v>390804.77</v>
       </c>
       <c r="D61" s="16"/>
       <c r="E61" s="7" t="str">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="C62" s="13" t="n">
         <f aca="false">'Targets 2027'!K9</f>
-        <v>425684.45</v>
+        <v>412075.95</v>
       </c>
       <c r="D62" s="16"/>
       <c r="E62" s="7" t="str">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="C63" s="13" t="n">
         <f aca="false">'Targets 2027'!L9</f>
-        <v>416009.75</v>
+        <v>402337.19</v>
       </c>
       <c r="D63" s="16"/>
       <c r="E63" s="7" t="str">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="C64" s="13" t="n">
         <f aca="false">'Targets 2027'!M9</f>
-        <v>453974.83</v>
+        <v>436438.26</v>
       </c>
       <c r="D64" s="16"/>
       <c r="E64" s="7" t="str">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="C65" s="13" t="n">
         <f aca="false">'Targets 2027'!B10</f>
-        <v>257347.15</v>
+        <v>249935.35</v>
       </c>
       <c r="D65" s="16"/>
       <c r="E65" s="7" t="str">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="C66" s="13" t="n">
         <f aca="false">'Targets 2027'!C10</f>
-        <v>234138.23</v>
+        <v>228766.86</v>
       </c>
       <c r="D66" s="16"/>
       <c r="E66" s="7" t="str">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="C67" s="13" t="n">
         <f aca="false">'Targets 2027'!D10</f>
-        <v>265056.56</v>
+        <v>260996.01</v>
       </c>
       <c r="D67" s="16"/>
       <c r="E67" s="7" t="str">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="C68" s="13" t="n">
         <f aca="false">'Targets 2027'!E10</f>
-        <v>262039.19</v>
+        <v>252237.93</v>
       </c>
       <c r="D68" s="16"/>
       <c r="E68" s="7" t="str">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="C69" s="13" t="n">
         <f aca="false">'Targets 2027'!F10</f>
-        <v>279695.99</v>
+        <v>273929.29</v>
       </c>
       <c r="D69" s="16"/>
       <c r="E69" s="7" t="str">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="C70" s="13" t="n">
         <f aca="false">'Targets 2027'!G10</f>
-        <v>254919.15</v>
+        <v>247214.98</v>
       </c>
       <c r="D70" s="16"/>
       <c r="E70" s="7" t="str">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C71" s="13" t="n">
         <f aca="false">'Targets 2027'!H10</f>
-        <v>278642.95</v>
+        <v>269489.88</v>
       </c>
       <c r="D71" s="16"/>
       <c r="E71" s="7" t="str">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="C72" s="13" t="n">
         <f aca="false">'Targets 2027'!I10</f>
-        <v>278428.66</v>
+        <v>274315.81</v>
       </c>
       <c r="D72" s="16"/>
       <c r="E72" s="7" t="str">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="C73" s="13" t="n">
         <f aca="false">'Targets 2027'!J10</f>
-        <v>244515.81</v>
+        <v>238484.98</v>
       </c>
       <c r="D73" s="16"/>
       <c r="E73" s="7" t="str">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="C74" s="13" t="n">
         <f aca="false">'Targets 2027'!K10</f>
-        <v>257847.21</v>
+        <v>252570.07</v>
       </c>
       <c r="D74" s="16"/>
       <c r="E74" s="7" t="str">
@@ -3591,7 +3591,7 @@
       </c>
       <c r="C75" s="13" t="n">
         <f aca="false">'Targets 2027'!L10</f>
-        <v>250121.21</v>
+        <v>244479.98</v>
       </c>
       <c r="D75" s="16"/>
       <c r="E75" s="7" t="str">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="C76" s="13" t="n">
         <f aca="false">'Targets 2027'!M10</f>
-        <v>264806</v>
+        <v>256922.52</v>
       </c>
       <c r="D76" s="16"/>
       <c r="E76" s="7" t="str">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C77" s="13" t="n">
         <f aca="false">'Targets 2027'!B11</f>
-        <v>70024.33</v>
+        <v>68962.29</v>
       </c>
       <c r="D77" s="16"/>
       <c r="E77" s="7" t="str">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="C78" s="13" t="n">
         <f aca="false">'Targets 2027'!C11</f>
-        <v>65363.47</v>
+        <v>64298.16</v>
       </c>
       <c r="D78" s="16"/>
       <c r="E78" s="7" t="str">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="C79" s="13" t="n">
         <f aca="false">'Targets 2027'!D11</f>
-        <v>80282.84</v>
+        <v>80750.82</v>
       </c>
       <c r="D79" s="16"/>
       <c r="E79" s="7" t="str">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="C80" s="13" t="n">
         <f aca="false">'Targets 2027'!E11</f>
-        <v>78691.41</v>
+        <v>76408.93</v>
       </c>
       <c r="D80" s="16"/>
       <c r="E80" s="7" t="str">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="C81" s="13" t="n">
         <f aca="false">'Targets 2027'!F11</f>
-        <v>81914.6</v>
+        <v>81062.97</v>
       </c>
       <c r="D81" s="16"/>
       <c r="E81" s="7" t="str">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="C82" s="13" t="n">
         <f aca="false">'Targets 2027'!G11</f>
-        <v>80680.83</v>
+        <v>79234.8</v>
       </c>
       <c r="D82" s="16"/>
       <c r="E82" s="7" t="str">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="C83" s="13" t="n">
         <f aca="false">'Targets 2027'!H11</f>
-        <v>95117.93</v>
+        <v>93765.52</v>
       </c>
       <c r="D83" s="16"/>
       <c r="E83" s="7" t="str">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="C84" s="13" t="n">
         <f aca="false">'Targets 2027'!I11</f>
-        <v>92412.44</v>
+        <v>92719.44</v>
       </c>
       <c r="D84" s="16"/>
       <c r="E84" s="7" t="str">
@@ -3801,7 +3801,7 @@
       </c>
       <c r="C85" s="13" t="n">
         <f aca="false">'Targets 2027'!J11</f>
-        <v>75560.91</v>
+        <v>73936.93</v>
       </c>
       <c r="D85" s="16"/>
       <c r="E85" s="7" t="str">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="C86" s="13" t="n">
         <f aca="false">'Targets 2027'!K11</f>
-        <v>74362.39</v>
+        <v>72624.46</v>
       </c>
       <c r="D86" s="16"/>
       <c r="E86" s="7" t="str">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="C87" s="13" t="n">
         <f aca="false">'Targets 2027'!L11</f>
-        <v>67804.32</v>
+        <v>66319.24</v>
       </c>
       <c r="D87" s="16"/>
       <c r="E87" s="7" t="str">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C88" s="13" t="n">
         <f aca="false">'Targets 2027'!M11</f>
-        <v>69510.22</v>
+        <v>67419.34</v>
       </c>
       <c r="D88" s="16"/>
       <c r="E88" s="7" t="str">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="C89" s="13" t="n">
         <f aca="false">'Targets 2027'!B12</f>
-        <v>296914.31</v>
+        <v>272028.46</v>
       </c>
       <c r="D89" s="16"/>
       <c r="E89" s="7" t="str">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="C90" s="13" t="n">
         <f aca="false">'Targets 2027'!C12</f>
-        <v>286294.25</v>
+        <v>262868.2</v>
       </c>
       <c r="D90" s="16"/>
       <c r="E90" s="7" t="str">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="C91" s="13" t="n">
         <f aca="false">'Targets 2027'!D12</f>
-        <v>338579.82</v>
+        <v>321610.48</v>
       </c>
       <c r="D91" s="16"/>
       <c r="E91" s="7" t="str">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="C92" s="13" t="n">
         <f aca="false">'Targets 2027'!E12</f>
-        <v>342033.7</v>
+        <v>321350.71</v>
       </c>
       <c r="D92" s="16"/>
       <c r="E92" s="7" t="str">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="C93" s="13" t="n">
         <f aca="false">'Targets 2027'!F12</f>
-        <v>347090.01</v>
+        <v>327929.65</v>
       </c>
       <c r="D93" s="16"/>
       <c r="E93" s="7" t="str">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="C94" s="13" t="n">
         <f aca="false">'Targets 2027'!G12</f>
-        <v>332147.99</v>
+        <v>311502.27</v>
       </c>
       <c r="D94" s="16"/>
       <c r="E94" s="7" t="str">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="C95" s="13" t="n">
         <f aca="false">'Targets 2027'!H12</f>
-        <v>367354.16</v>
+        <v>345099.66</v>
       </c>
       <c r="D95" s="16"/>
       <c r="E95" s="7" t="str">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="C96" s="13" t="n">
         <f aca="false">'Targets 2027'!I12</f>
-        <v>368327.3</v>
+        <v>352910.33</v>
       </c>
       <c r="D96" s="16"/>
       <c r="E96" s="7" t="str">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="C97" s="13" t="n">
         <f aca="false">'Targets 2027'!J12</f>
-        <v>307233.84</v>
+        <v>290355.8</v>
       </c>
       <c r="D97" s="16"/>
       <c r="E97" s="7" t="str">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="C98" s="13" t="n">
         <f aca="false">'Targets 2027'!K12</f>
-        <v>316289.17</v>
+        <v>299061.64</v>
       </c>
       <c r="D98" s="16"/>
       <c r="E98" s="7" t="str">
@@ -4095,7 +4095,7 @@
       </c>
       <c r="C99" s="13" t="n">
         <f aca="false">'Targets 2027'!L12</f>
-        <v>306667.72</v>
+        <v>289356.18</v>
       </c>
       <c r="D99" s="16"/>
       <c r="E99" s="7" t="str">
@@ -4116,7 +4116,7 @@
       </c>
       <c r="C100" s="13" t="n">
         <f aca="false">'Targets 2027'!M12</f>
-        <v>319163.66</v>
+        <v>296212.08</v>
       </c>
       <c r="D100" s="16"/>
       <c r="E100" s="7" t="str">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="C101" s="13" t="n">
         <f aca="false">'Targets 2027'!B13</f>
-        <v>327146.38</v>
+        <v>310339.79</v>
       </c>
       <c r="D101" s="16"/>
       <c r="E101" s="7" t="str">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C102" s="13" t="n">
         <f aca="false">'Targets 2027'!C13</f>
-        <v>271492.7</v>
+        <v>261447.34</v>
       </c>
       <c r="D102" s="16"/>
       <c r="E102" s="7" t="str">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="C103" s="13" t="n">
         <f aca="false">'Targets 2027'!D13</f>
-        <v>316609.81</v>
+        <v>310773.11</v>
       </c>
       <c r="D103" s="16"/>
       <c r="E103" s="7" t="str">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="C104" s="13" t="n">
         <f aca="false">'Targets 2027'!E13</f>
-        <v>307133.63</v>
+        <v>296667.43</v>
       </c>
       <c r="D104" s="16"/>
       <c r="E104" s="7" t="str">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="C105" s="13" t="n">
         <f aca="false">'Targets 2027'!F13</f>
-        <v>349631.07</v>
+        <v>339151.24</v>
       </c>
       <c r="D105" s="16"/>
       <c r="E105" s="7" t="str">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="C106" s="13" t="n">
         <f aca="false">'Targets 2027'!G13</f>
-        <v>326325.44</v>
+        <v>316744.84</v>
       </c>
       <c r="D106" s="16"/>
       <c r="E106" s="7" t="str">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="C107" s="13" t="n">
         <f aca="false">'Targets 2027'!H13</f>
-        <v>363061.05</v>
+        <v>349578</v>
       </c>
       <c r="D107" s="16"/>
       <c r="E107" s="7" t="str">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="C108" s="13" t="n">
         <f aca="false">'Targets 2027'!I13</f>
-        <v>359674.68</v>
+        <v>352910.43</v>
       </c>
       <c r="D108" s="16"/>
       <c r="E108" s="7" t="str">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="C109" s="13" t="n">
         <f aca="false">'Targets 2027'!J13</f>
-        <v>296046.26</v>
+        <v>285576.59</v>
       </c>
       <c r="D109" s="16"/>
       <c r="E109" s="7" t="str">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="C110" s="13" t="n">
         <f aca="false">'Targets 2027'!K13</f>
-        <v>317470.65</v>
+        <v>300807.14</v>
       </c>
       <c r="D110" s="16"/>
       <c r="E110" s="7" t="str">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="C111" s="13" t="n">
         <f aca="false">'Targets 2027'!L13</f>
-        <v>297737.89</v>
+        <v>287803.85</v>
       </c>
       <c r="D111" s="16"/>
       <c r="E111" s="7" t="str">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="C112" s="13" t="n">
         <f aca="false">'Targets 2027'!M13</f>
-        <v>322139.38</v>
+        <v>306150.86</v>
       </c>
       <c r="D112" s="16"/>
       <c r="E112" s="7" t="str">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="C113" s="13" t="n">
         <f aca="false">'Targets 2027'!B15</f>
-        <v>49132.16</v>
+        <v>48441.74</v>
       </c>
       <c r="D113" s="16"/>
       <c r="E113" s="7" t="str">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="C114" s="13" t="n">
         <f aca="false">'Targets 2027'!C15</f>
-        <v>47789.29</v>
+        <v>47416.51</v>
       </c>
       <c r="D114" s="16"/>
       <c r="E114" s="7" t="str">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="C115" s="13" t="n">
         <f aca="false">'Targets 2027'!D15</f>
-        <v>57042.34</v>
+        <v>56982.27</v>
       </c>
       <c r="D115" s="16"/>
       <c r="E115" s="7" t="str">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="C116" s="13" t="n">
         <f aca="false">'Targets 2027'!E15</f>
-        <v>58246.45</v>
+        <v>57181.59</v>
       </c>
       <c r="D116" s="16"/>
       <c r="E116" s="7" t="str">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="C117" s="13" t="n">
         <f aca="false">'Targets 2027'!F15</f>
-        <v>61613.98</v>
+        <v>60086.27</v>
       </c>
       <c r="D117" s="16"/>
       <c r="E117" s="7" t="str">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="C118" s="13" t="n">
         <f aca="false">'Targets 2027'!G15</f>
-        <v>59373.16</v>
+        <v>57726</v>
       </c>
       <c r="D118" s="16"/>
       <c r="E118" s="7" t="str">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="C119" s="13" t="n">
         <f aca="false">'Targets 2027'!H15</f>
-        <v>69005.96</v>
+        <v>66755.21</v>
       </c>
       <c r="D119" s="16"/>
       <c r="E119" s="7" t="str">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="C120" s="13" t="n">
         <f aca="false">'Targets 2027'!I15</f>
-        <v>63974.68</v>
+        <v>62712.99</v>
       </c>
       <c r="D120" s="16"/>
       <c r="E120" s="7" t="str">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="C121" s="13" t="n">
         <f aca="false">'Targets 2027'!J15</f>
-        <v>55593.97</v>
+        <v>54320.07</v>
       </c>
       <c r="D121" s="16"/>
       <c r="E121" s="7" t="str">
@@ -4712,11 +4712,11 @@
       </c>
       <c r="G5" s="13" t="n">
         <f aca="false">'Targets 2027'!R5</f>
-        <v>3119407.01</v>
+        <v>2939876.01</v>
       </c>
       <c r="H5" s="7" t="n">
         <f aca="false">G5-E5</f>
-        <v>361651.2</v>
+        <v>182120.2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4740,11 +4740,11 @@
       </c>
       <c r="G6" s="13" t="n">
         <f aca="false">'Targets 2027'!R6</f>
-        <v>2641664.44</v>
+        <v>2523110.65</v>
       </c>
       <c r="H6" s="7" t="n">
         <f aca="false">G6-E6</f>
-        <v>277730.830000001</v>
+        <v>159177.04</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4768,11 +4768,11 @@
       </c>
       <c r="G7" s="13" t="n">
         <f aca="false">'Targets 2027'!R7</f>
-        <v>4233666.85</v>
+        <v>4055158.57</v>
       </c>
       <c r="H7" s="7" t="n">
         <f aca="false">G7-E7</f>
-        <v>425903.09</v>
+        <v>247394.81</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4796,11 +4796,11 @@
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">'Targets 2027'!R8</f>
-        <v>4307690.71</v>
+        <v>4195611.3</v>
       </c>
       <c r="H8" s="7" t="n">
         <f aca="false">G8-E8</f>
-        <v>173193.33</v>
+        <v>61113.9199999999</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4824,11 +4824,11 @@
       </c>
       <c r="G9" s="13" t="n">
         <f aca="false">'Targets 2027'!R9</f>
-        <v>5151283.7</v>
+        <v>4981365.48</v>
       </c>
       <c r="H9" s="7" t="n">
         <f aca="false">G9-E9</f>
-        <v>441405.5</v>
+        <v>271487.279999999</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4852,11 +4852,11 @@
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">'Targets 2027'!R10</f>
-        <v>3127558.11</v>
+        <v>3049343.66</v>
       </c>
       <c r="H10" s="7" t="n">
         <f aca="false">G10-E10</f>
-        <v>85804.9099999997</v>
+        <v>7590.45999999996</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">'Targets 2027'!R11</f>
-        <v>931725.69</v>
+        <v>917502.9</v>
       </c>
       <c r="H11" s="7" t="n">
         <f aca="false">G11-E11</f>
-        <v>-5046.27000000002</v>
+        <v>-19269.0599999999</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">'Targets 2027'!R12</f>
-        <v>3928095.93</v>
+        <v>3690285.46</v>
       </c>
       <c r="H12" s="7" t="n">
         <f aca="false">G12-E12</f>
-        <v>469572.37</v>
+        <v>231761.9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4936,11 +4936,11 @@
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">'Targets 2027'!R13</f>
-        <v>3854468.94</v>
+        <v>3717950.62</v>
       </c>
       <c r="H13" s="7" t="n">
         <f aca="false">G13-E13</f>
-        <v>247474.57</v>
+        <v>110956.25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4964,11 +4964,11 @@
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">'Targets 2027'!R15</f>
-        <v>896771.99</v>
+        <v>886622.65</v>
       </c>
       <c r="H14" s="7" t="n">
         <f aca="false">G14-E14</f>
-        <v>29012.87</v>
+        <v>18863.53</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4997,11 +4997,11 @@
       </c>
       <c r="G15" s="10" t="n">
         <f aca="false">SUM(G5:G14)</f>
-        <v>32192333.37</v>
+        <v>30956827.3</v>
       </c>
       <c r="H15" s="10" t="n">
         <f aca="false">SUM(H5:H14)</f>
-        <v>2506702.4</v>
+        <v>1271196.33</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Apply management adjustments to the run-rate and the 2027 targets
Run-rate 2027 for three cafés is set on the 2026 finish instead of their
last 45 days alone: Coronado +1.2% (reads -1.5%), La Jolla Juicery +1.5%
(-1.2%) and Newport Beach +1.9% (+0.6%). Every 2027 month moves by one
factor, so the seasons and the 2026 finish stay as they were. Each page
notes the adjustment, and the method, 2027 and definitions pages say so.

Targets keep 65% of the plan's growth and add points of growth on 2026 to
every month: the three cafés above get the points their run-rate was raised
(+2.7, +2.7, +1.3), La Jolla Café +3, and Beverly Hills is set 5 points
over its run-rate (+3.4). The nine come to $30.42M (+9.4% on 2026), $31.31M
with La Jolla Cove; the nine's run-rate is $28.89M (+0.2% on the budget).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C2c9kVN8V8siaKQgSRcGwk
</commit_message>
<xml_diff>
--- a/outputs/Parakeet_2027_Manager_Targets.xlsx
+++ b/outputs/Parakeet_2027_Manager_Targets.xlsx
@@ -45,12 +45,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="64">
   <si>
     <t xml:space="preserve">Parakeet Café · 2027 sales targets by store</t>
   </si>
   <si>
-    <t xml:space="preserve">Net sales targets per month (each month of 2026 plus 65% of the growth in our plan; La Jolla Cove switches to the budget's remodeled rate from its Oct 1, 2027 reopening). Blue = values from the analysis; black = formulas.</t>
+    <t xml:space="preserve">Net sales targets per month (each month of 2026 plus 65% of the growth in our plan, raised by management for five cafés: see 'Reference'; La Jolla Cove switches to the budget's remodeled rate from its Oct 1, 2027 reopening). Blue = values from the analysis; black = formulas.</t>
   </si>
   <si>
     <t xml:space="preserve">Store</t>
@@ -209,7 +209,7 @@
     <t xml:space="preserve">Reference: 2026 finish and 2027 under each view</t>
   </si>
   <si>
-    <t xml:space="preserve">Sources: Toast POS net sales through Oct 14, 2026; investor budget workbook (2027_Sales_budget_Investors.xlsx); run-rate = last 45 days seasonally adjusted; target = each month of 2026 plus 65% of the growth in our plan.</t>
+    <t xml:space="preserve">Sources: Toast POS net sales through Oct 14, 2026; investor budget workbook (2027_Sales_budget_Investors.xlsx); run-rate = last 45 days seasonally adjusted; target = each month of 2026 plus 65% of the growth in our plan; management adjustments below.</t>
   </si>
   <si>
     <t xml:space="preserve">2025 actual (Toast)</t>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t xml:space="preserve">La Jolla Cove's run-rate objective and target include the budget's remodeled $125K a month from Oct 1, 2027. New cafés are not included.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management adjustments (October 2026). Run-rate 2027 set to Coronado +1.2%, La Jolla Juicery +1.5% and Newport Beach +1.9% on 2026 (the last 45 days alone: −1.5%, −1.2% and +0.6%). Targets, in points of growth on 2026: Coronado, La Jolla Juicery and Newport Beach get the points their run-rate was raised (+2.7, +2.7 and +1.3); La Jolla Café 3 points more; Beverly Hills is set 5 points over its run-rate (+3.4).</t>
   </si>
 </sst>
 </file>
@@ -789,67 +792,67 @@
         <v>22</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>222665.72</v>
+        <v>229043.04</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>215270.61</v>
+        <v>221446.69</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>237349.22</v>
+        <v>244072.04</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>230307.13</v>
+        <v>236927.79</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>255311.3</v>
+        <v>262818.69</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>248397</v>
+        <v>255781.63</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>255876.37</v>
+        <v>263640.32</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>267229.53</v>
+        <v>275300.19</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>241289.02</v>
+        <v>248448.85</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>259364.53</v>
+        <v>267705.91</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>255086.19</v>
+        <v>262923.86</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>251729.39</v>
+        <v>259321.32</v>
       </c>
       <c r="N5" s="7" t="n">
         <f aca="false">SUM(B5:D5)</f>
-        <v>675285.55</v>
+        <v>694561.77</v>
       </c>
       <c r="O5" s="7" t="n">
         <f aca="false">SUM(E5:G5)</f>
-        <v>734015.43</v>
+        <v>755528.11</v>
       </c>
       <c r="P5" s="7" t="n">
         <f aca="false">SUM(H5:J5)</f>
-        <v>764394.92</v>
+        <v>787389.36</v>
       </c>
       <c r="Q5" s="7" t="n">
         <f aca="false">SUM(K5:M5)</f>
-        <v>766180.11</v>
+        <v>789951.09</v>
       </c>
       <c r="R5" s="7" t="n">
         <f aca="false">SUM(B5:M5)</f>
-        <v>2939876.01</v>
+        <v>3027430.33</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>2606461.36</v>
       </c>
       <c r="T5" s="8" t="n">
         <f aca="false">IF(S5=0,"",R5/S5-1)</f>
-        <v>0.127918508640389</v>
+        <v>0.161509768170897</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -993,67 +996,67 @@
         <v>25</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>304631.98</v>
+        <v>312346.91</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>275671.13</v>
+        <v>282707.15</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>364481.8</v>
+        <v>374277.35</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>347969.67</v>
+        <v>356778.22</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>373536.14</v>
+        <v>383300.65</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>366821.39</v>
+        <v>376007.58</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>499555.29</v>
+        <v>511998.59</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>418224.45</v>
+        <v>428895.84</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>301447.17</v>
+        <v>309013.05</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>312304.44</v>
+        <v>319848.01</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>296489.07</v>
+        <v>303872.93</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>334478.77</v>
+        <v>342568.81</v>
       </c>
       <c r="N8" s="7" t="n">
         <f aca="false">SUM(B8:D8)</f>
-        <v>944784.91</v>
+        <v>969331.41</v>
       </c>
       <c r="O8" s="7" t="n">
         <f aca="false">SUM(E8:G8)</f>
-        <v>1088327.2</v>
+        <v>1116086.45</v>
       </c>
       <c r="P8" s="7" t="n">
         <f aca="false">SUM(H8:J8)</f>
-        <v>1219226.91</v>
+        <v>1249907.48</v>
       </c>
       <c r="Q8" s="7" t="n">
         <f aca="false">SUM(K8:M8)</f>
-        <v>943272.28</v>
+        <v>966289.75</v>
       </c>
       <c r="R8" s="7" t="n">
         <f aca="false">SUM(B8:M8)</f>
-        <v>4195611.3</v>
+        <v>4301615.09</v>
       </c>
       <c r="S8" s="6" t="n">
         <v>3987463.81</v>
       </c>
       <c r="T8" s="8" t="n">
         <f aca="false">IF(S8=0,"",R8/S8-1)</f>
-        <v>0.0522004712564399</v>
+        <v>0.0787847351020847</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1129,67 +1132,67 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>249935.35</v>
+        <v>257020.47</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>228766.86</v>
+        <v>235330.6</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>260996.01</v>
+        <v>268599.66</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>252237.93</v>
+        <v>259259</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>273929.29</v>
+        <v>281825.88</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>247214.98</v>
+        <v>254202.2</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>269489.88</v>
+        <v>277064.62</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>274315.81</v>
+        <v>282316.14</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>238484.98</v>
+        <v>245303.53</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>252570.07</v>
+        <v>259853.16</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>244479.98</v>
+        <v>251500.08</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>256922.52</v>
+        <v>264190.98</v>
       </c>
       <c r="N10" s="7" t="n">
         <f aca="false">SUM(B10:D10)</f>
-        <v>739698.22</v>
+        <v>760950.73</v>
       </c>
       <c r="O10" s="7" t="n">
         <f aca="false">SUM(E10:G10)</f>
-        <v>773382.2</v>
+        <v>795287.08</v>
       </c>
       <c r="P10" s="7" t="n">
         <f aca="false">SUM(H10:J10)</f>
-        <v>782290.67</v>
+        <v>804684.29</v>
       </c>
       <c r="Q10" s="7" t="n">
         <f aca="false">SUM(K10:M10)</f>
-        <v>753972.57</v>
+        <v>775544.22</v>
       </c>
       <c r="R10" s="7" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>3049343.66</v>
+        <v>3136466.32</v>
       </c>
       <c r="S10" s="6" t="n">
         <v>2904088.3</v>
       </c>
       <c r="T10" s="8" t="n">
         <f aca="false">IF(S10=0,"",R10/S10-1)</f>
-        <v>0.0500175425106737</v>
+        <v>0.0800175462984374</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1197,67 +1200,67 @@
         <v>28</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>68962.29</v>
+        <v>70800.15</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>64298.16</v>
+        <v>66007.9</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>80750.82</v>
+        <v>82990.05</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>76408.93</v>
+        <v>78388.91</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>81062.97</v>
+        <v>83243.53</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>79234.8</v>
+        <v>81334.93</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>93765.52</v>
+        <v>96269.06</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>92719.44</v>
+        <v>95278.83</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>73936.93</v>
+        <v>75882.64</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>72624.46</v>
+        <v>74528.35</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>66319.24</v>
+        <v>68063.03</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>67419.34</v>
+        <v>69162.45</v>
       </c>
       <c r="N11" s="7" t="n">
         <f aca="false">SUM(B11:D11)</f>
-        <v>214011.27</v>
+        <v>219798.1</v>
       </c>
       <c r="O11" s="7" t="n">
         <f aca="false">SUM(E11:G11)</f>
-        <v>236706.7</v>
+        <v>242967.37</v>
       </c>
       <c r="P11" s="7" t="n">
         <f aca="false">SUM(H11:J11)</f>
-        <v>260421.89</v>
+        <v>267430.53</v>
       </c>
       <c r="Q11" s="7" t="n">
         <f aca="false">SUM(K11:M11)</f>
-        <v>206363.04</v>
+        <v>211753.83</v>
       </c>
       <c r="R11" s="7" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>917502.9</v>
+        <v>941949.83</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>891089.16</v>
       </c>
       <c r="T11" s="8" t="n">
         <f aca="false">IF(S11=0,"",R11/S11-1)</f>
-        <v>0.0296420843005205</v>
+        <v>0.057076970838698</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1333,67 +1336,67 @@
         <v>30</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>310339.79</v>
+        <v>313961.18</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>261447.34</v>
+        <v>264597.31</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>310773.11</v>
+        <v>314664.44</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>296667.43</v>
+        <v>300264.21</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>339151.24</v>
+        <v>343298.88</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>316744.84</v>
+        <v>320623.44</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>349578</v>
+        <v>353788.55</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>352910.43</v>
+        <v>357326.1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>285576.59</v>
+        <v>289029.4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>300807.14</v>
+        <v>304308.3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>287803.85</v>
+        <v>291298.45</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>306150.86</v>
+        <v>309737.62</v>
       </c>
       <c r="N13" s="7" t="n">
         <f aca="false">SUM(B13:D13)</f>
-        <v>882560.24</v>
+        <v>893222.93</v>
       </c>
       <c r="O13" s="7" t="n">
         <f aca="false">SUM(E13:G13)</f>
-        <v>952563.51</v>
+        <v>964186.53</v>
       </c>
       <c r="P13" s="7" t="n">
         <f aca="false">SUM(H13:J13)</f>
-        <v>988065.02</v>
+        <v>1000144.05</v>
       </c>
       <c r="Q13" s="7" t="n">
         <f aca="false">SUM(K13:M13)</f>
-        <v>894761.85</v>
+        <v>905344.37</v>
       </c>
       <c r="R13" s="7" t="n">
         <f aca="false">SUM(B13:M13)</f>
-        <v>3717950.62</v>
+        <v>3762897.88</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>3464416.6</v>
       </c>
       <c r="T13" s="8" t="n">
         <f aca="false">IF(S13=0,"",R13/S13-1)</f>
-        <v>0.0731823130047349</v>
+        <v>0.0861562896332964</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1402,71 +1405,71 @@
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">SUM(B5:B13)</f>
-        <v>2391694.17</v>
+        <v>2418330.79</v>
       </c>
       <c r="C14" s="10" t="n">
         <f aca="false">SUM(C5:C13)</f>
-        <v>2167452.91</v>
+        <v>2192088.46</v>
       </c>
       <c r="D14" s="10" t="n">
         <f aca="false">SUM(D5:D13)</f>
-        <v>2555971.52</v>
+        <v>2586224.1</v>
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">SUM(E5:E13)</f>
-        <v>2473977.92</v>
+        <v>2502004.96</v>
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">SUM(F5:F13)</f>
-        <v>2677385.31</v>
+        <v>2708882</v>
       </c>
       <c r="G14" s="10" t="n">
         <f aca="false">SUM(G5:G13)</f>
-        <v>2505024.89</v>
+        <v>2534561.66</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">SUM(H5:H13)</f>
-        <v>2785046.12</v>
+        <v>2819542.2</v>
       </c>
       <c r="I14" s="10" t="n">
         <f aca="false">SUM(I5:I13)</f>
-        <v>2767746.03</v>
+        <v>2801463.47</v>
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">SUM(J5:J13)</f>
-        <v>2340472.77</v>
+        <v>2367415.55</v>
       </c>
       <c r="K14" s="10" t="n">
         <f aca="false">SUM(K5:K13)</f>
-        <v>2461357.09</v>
+        <v>2489930.18</v>
       </c>
       <c r="L14" s="10" t="n">
         <f aca="false">SUM(L5:L13)</f>
-        <v>2409557.34</v>
+        <v>2437037.36</v>
       </c>
       <c r="M14" s="10" t="n">
         <f aca="false">SUM(M5:M13)</f>
-        <v>2534518.58</v>
+        <v>2562798.88</v>
       </c>
       <c r="N14" s="10" t="n">
         <f aca="false">SUM(N5:N13)</f>
-        <v>7115118.6</v>
+        <v>7196643.35</v>
       </c>
       <c r="O14" s="10" t="n">
         <f aca="false">SUM(O5:O13)</f>
-        <v>7656388.12</v>
+        <v>7745448.62</v>
       </c>
       <c r="P14" s="10" t="n">
         <f aca="false">SUM(P5:P13)</f>
-        <v>7893264.92</v>
+        <v>7988421.22</v>
       </c>
       <c r="Q14" s="10" t="n">
         <f aca="false">SUM(Q5:Q13)</f>
-        <v>7405433.01</v>
+        <v>7489766.42</v>
       </c>
       <c r="R14" s="10" t="n">
         <f aca="false">SUM(R5:R13)</f>
-        <v>30070204.65</v>
+        <v>30420279.61</v>
       </c>
       <c r="S14" s="10" t="n">
         <f aca="false">SUM(S5:S13)</f>
@@ -1474,7 +1477,7 @@
       </c>
       <c r="T14" s="11" t="n">
         <f aca="false">IF(S14=0,"",R14/S14-1)</f>
-        <v>0.0818744350170033</v>
+        <v>0.0944695321894995</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1551,71 +1554,71 @@
       </c>
       <c r="B16" s="10" t="n">
         <f aca="false">B14+B15</f>
-        <v>2440135.91</v>
+        <v>2466772.53</v>
       </c>
       <c r="C16" s="10" t="n">
         <f aca="false">C14+C15</f>
-        <v>2214869.42</v>
+        <v>2239504.97</v>
       </c>
       <c r="D16" s="10" t="n">
         <f aca="false">D14+D15</f>
-        <v>2612953.79</v>
+        <v>2643206.37</v>
       </c>
       <c r="E16" s="10" t="n">
         <f aca="false">E14+E15</f>
-        <v>2531159.51</v>
+        <v>2559186.55</v>
       </c>
       <c r="F16" s="10" t="n">
         <f aca="false">F14+F15</f>
-        <v>2737471.58</v>
+        <v>2768968.27</v>
       </c>
       <c r="G16" s="10" t="n">
         <f aca="false">G14+G15</f>
-        <v>2562750.89</v>
+        <v>2592287.66</v>
       </c>
       <c r="H16" s="10" t="n">
         <f aca="false">H14+H15</f>
-        <v>2851801.33</v>
+        <v>2886297.41</v>
       </c>
       <c r="I16" s="10" t="n">
         <f aca="false">I14+I15</f>
-        <v>2830459.02</v>
+        <v>2864176.46</v>
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">J14+J15</f>
-        <v>2394792.84</v>
+        <v>2421735.62</v>
       </c>
       <c r="K16" s="10" t="n">
         <f aca="false">K14+K15</f>
-        <v>2586357.09</v>
+        <v>2614930.18</v>
       </c>
       <c r="L16" s="10" t="n">
         <f aca="false">L14+L15</f>
-        <v>2534557.34</v>
+        <v>2562037.36</v>
       </c>
       <c r="M16" s="10" t="n">
         <f aca="false">M14+M15</f>
-        <v>2659518.58</v>
+        <v>2687798.88</v>
       </c>
       <c r="N16" s="10" t="n">
         <f aca="false">N14+N15</f>
-        <v>7267959.12</v>
+        <v>7349483.87</v>
       </c>
       <c r="O16" s="10" t="n">
         <f aca="false">O14+O15</f>
-        <v>7831381.98</v>
+        <v>7920442.48</v>
       </c>
       <c r="P16" s="10" t="n">
         <f aca="false">P14+P15</f>
-        <v>8077053.19</v>
+        <v>8172209.49</v>
       </c>
       <c r="Q16" s="10" t="n">
         <f aca="false">Q14+Q15</f>
-        <v>7780433.01</v>
+        <v>7864766.42</v>
       </c>
       <c r="R16" s="10" t="n">
         <f aca="false">R14+R15</f>
-        <v>30956827.3</v>
+        <v>31306902.26</v>
       </c>
       <c r="S16" s="10" t="n">
         <f aca="false">S14+S15</f>
@@ -1623,7 +1626,7 @@
       </c>
       <c r="T16" s="11" t="n">
         <f aca="false">IF(S16=0,"",R16/S16-1)</f>
-        <v>0.0888539417243652</v>
+        <v>0.101167235215362</v>
       </c>
     </row>
   </sheetData>
@@ -1689,7 +1692,7 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">'Targets 2027'!R5</f>
-        <v>2939876.01</v>
+        <v>3027430.33</v>
       </c>
       <c r="C5" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A5,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1776,7 +1779,7 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">'Targets 2027'!R8</f>
-        <v>4195611.3</v>
+        <v>4301615.09</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A8,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1834,7 +1837,7 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">'Targets 2027'!R10</f>
-        <v>3049343.66</v>
+        <v>3136466.32</v>
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A10,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1863,7 +1866,7 @@
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">'Targets 2027'!R11</f>
-        <v>917502.9</v>
+        <v>941949.83</v>
       </c>
       <c r="C11" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A11,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1921,7 +1924,7 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">'Targets 2027'!R13</f>
-        <v>3717950.62</v>
+        <v>3762897.88</v>
       </c>
       <c r="C13" s="7" t="n">
         <f aca="false">SUMIFS('Monthly tracking'!$C$5:$C$124,'Monthly tracking'!$A$5:$A$124,A13,'Monthly tracking'!$D$5:$D$124,"&lt;&gt;")</f>
@@ -1979,7 +1982,7 @@
       </c>
       <c r="B15" s="10" t="n">
         <f aca="false">SUM(B5:B14)</f>
-        <v>30956827.3</v>
+        <v>31306902.26</v>
       </c>
       <c r="C15" s="10" t="n">
         <f aca="false">SUM(C5:C14)</f>
@@ -2067,7 +2070,7 @@
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">'Targets 2027'!B5</f>
-        <v>222665.72</v>
+        <v>229043.04</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="7" t="str">
@@ -2091,7 +2094,7 @@
       </c>
       <c r="C6" s="13" t="n">
         <f aca="false">'Targets 2027'!C5</f>
-        <v>215270.61</v>
+        <v>221446.69</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="7" t="str">
@@ -2115,7 +2118,7 @@
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">'Targets 2027'!D5</f>
-        <v>237349.22</v>
+        <v>244072.04</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="7" t="str">
@@ -2139,7 +2142,7 @@
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">'Targets 2027'!E5</f>
-        <v>230307.13</v>
+        <v>236927.79</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="7" t="str">
@@ -2163,7 +2166,7 @@
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">'Targets 2027'!F5</f>
-        <v>255311.3</v>
+        <v>262818.69</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="7" t="str">
@@ -2184,7 +2187,7 @@
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">'Targets 2027'!G5</f>
-        <v>248397</v>
+        <v>255781.63</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="7" t="str">
@@ -2208,7 +2211,7 @@
       </c>
       <c r="C11" s="13" t="n">
         <f aca="false">'Targets 2027'!H5</f>
-        <v>255876.37</v>
+        <v>263640.32</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="7" t="str">
@@ -2247,7 +2250,7 @@
       </c>
       <c r="C12" s="13" t="n">
         <f aca="false">'Targets 2027'!I5</f>
-        <v>267229.53</v>
+        <v>275300.19</v>
       </c>
       <c r="D12" s="16"/>
       <c r="E12" s="7" t="str">
@@ -2266,18 +2269,18 @@
       </c>
       <c r="J12" s="13" t="n">
         <f aca="false">C5</f>
-        <v>222665.72</v>
+        <v>229043.04</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>227000</v>
+        <v>234000</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(K12="","",K12-J12)</f>
-        <v>4334.28</v>
+        <v>4956.95999999999</v>
       </c>
       <c r="M12" s="8" t="n">
         <f aca="false">IF(K12="","",K12/J12-1)</f>
-        <v>0.0194654120984585</v>
+        <v>0.0216420459665572</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2289,7 +2292,7 @@
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">'Targets 2027'!J5</f>
-        <v>241289.02</v>
+        <v>248448.85</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="7" t="str">
@@ -2310,7 +2313,7 @@
       </c>
       <c r="C14" s="13" t="n">
         <f aca="false">'Targets 2027'!K5</f>
-        <v>259364.53</v>
+        <v>267705.91</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="7" t="str">
@@ -2331,7 +2334,7 @@
       </c>
       <c r="C15" s="13" t="n">
         <f aca="false">'Targets 2027'!L5</f>
-        <v>255086.19</v>
+        <v>262923.86</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="7" t="str">
@@ -2352,7 +2355,7 @@
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">'Targets 2027'!M5</f>
-        <v>251729.39</v>
+        <v>259321.32</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="7" t="str">
@@ -2877,7 +2880,7 @@
       </c>
       <c r="C41" s="13" t="n">
         <f aca="false">'Targets 2027'!B8</f>
-        <v>304631.98</v>
+        <v>312346.91</v>
       </c>
       <c r="D41" s="16"/>
       <c r="E41" s="7" t="str">
@@ -2898,7 +2901,7 @@
       </c>
       <c r="C42" s="13" t="n">
         <f aca="false">'Targets 2027'!C8</f>
-        <v>275671.13</v>
+        <v>282707.15</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="7" t="str">
@@ -2919,7 +2922,7 @@
       </c>
       <c r="C43" s="13" t="n">
         <f aca="false">'Targets 2027'!D8</f>
-        <v>364481.8</v>
+        <v>374277.35</v>
       </c>
       <c r="D43" s="16"/>
       <c r="E43" s="7" t="str">
@@ -2940,7 +2943,7 @@
       </c>
       <c r="C44" s="13" t="n">
         <f aca="false">'Targets 2027'!E8</f>
-        <v>347969.67</v>
+        <v>356778.22</v>
       </c>
       <c r="D44" s="16"/>
       <c r="E44" s="7" t="str">
@@ -2961,7 +2964,7 @@
       </c>
       <c r="C45" s="13" t="n">
         <f aca="false">'Targets 2027'!F8</f>
-        <v>373536.14</v>
+        <v>383300.65</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="7" t="str">
@@ -2982,7 +2985,7 @@
       </c>
       <c r="C46" s="13" t="n">
         <f aca="false">'Targets 2027'!G8</f>
-        <v>366821.39</v>
+        <v>376007.58</v>
       </c>
       <c r="D46" s="16"/>
       <c r="E46" s="7" t="str">
@@ -3003,7 +3006,7 @@
       </c>
       <c r="C47" s="13" t="n">
         <f aca="false">'Targets 2027'!H8</f>
-        <v>499555.29</v>
+        <v>511998.59</v>
       </c>
       <c r="D47" s="16"/>
       <c r="E47" s="7" t="str">
@@ -3024,7 +3027,7 @@
       </c>
       <c r="C48" s="13" t="n">
         <f aca="false">'Targets 2027'!I8</f>
-        <v>418224.45</v>
+        <v>428895.84</v>
       </c>
       <c r="D48" s="16"/>
       <c r="E48" s="7" t="str">
@@ -3045,7 +3048,7 @@
       </c>
       <c r="C49" s="13" t="n">
         <f aca="false">'Targets 2027'!J8</f>
-        <v>301447.17</v>
+        <v>309013.05</v>
       </c>
       <c r="D49" s="16"/>
       <c r="E49" s="7" t="str">
@@ -3066,7 +3069,7 @@
       </c>
       <c r="C50" s="13" t="n">
         <f aca="false">'Targets 2027'!K8</f>
-        <v>312304.44</v>
+        <v>319848.01</v>
       </c>
       <c r="D50" s="16"/>
       <c r="E50" s="7" t="str">
@@ -3087,7 +3090,7 @@
       </c>
       <c r="C51" s="13" t="n">
         <f aca="false">'Targets 2027'!L8</f>
-        <v>296489.07</v>
+        <v>303872.93</v>
       </c>
       <c r="D51" s="16"/>
       <c r="E51" s="7" t="str">
@@ -3108,7 +3111,7 @@
       </c>
       <c r="C52" s="13" t="n">
         <f aca="false">'Targets 2027'!M8</f>
-        <v>334478.77</v>
+        <v>342568.81</v>
       </c>
       <c r="D52" s="16"/>
       <c r="E52" s="7" t="str">
@@ -3381,7 +3384,7 @@
       </c>
       <c r="C65" s="13" t="n">
         <f aca="false">'Targets 2027'!B10</f>
-        <v>249935.35</v>
+        <v>257020.47</v>
       </c>
       <c r="D65" s="16"/>
       <c r="E65" s="7" t="str">
@@ -3402,7 +3405,7 @@
       </c>
       <c r="C66" s="13" t="n">
         <f aca="false">'Targets 2027'!C10</f>
-        <v>228766.86</v>
+        <v>235330.6</v>
       </c>
       <c r="D66" s="16"/>
       <c r="E66" s="7" t="str">
@@ -3423,7 +3426,7 @@
       </c>
       <c r="C67" s="13" t="n">
         <f aca="false">'Targets 2027'!D10</f>
-        <v>260996.01</v>
+        <v>268599.66</v>
       </c>
       <c r="D67" s="16"/>
       <c r="E67" s="7" t="str">
@@ -3444,7 +3447,7 @@
       </c>
       <c r="C68" s="13" t="n">
         <f aca="false">'Targets 2027'!E10</f>
-        <v>252237.93</v>
+        <v>259259</v>
       </c>
       <c r="D68" s="16"/>
       <c r="E68" s="7" t="str">
@@ -3465,7 +3468,7 @@
       </c>
       <c r="C69" s="13" t="n">
         <f aca="false">'Targets 2027'!F10</f>
-        <v>273929.29</v>
+        <v>281825.88</v>
       </c>
       <c r="D69" s="16"/>
       <c r="E69" s="7" t="str">
@@ -3486,7 +3489,7 @@
       </c>
       <c r="C70" s="13" t="n">
         <f aca="false">'Targets 2027'!G10</f>
-        <v>247214.98</v>
+        <v>254202.2</v>
       </c>
       <c r="D70" s="16"/>
       <c r="E70" s="7" t="str">
@@ -3507,7 +3510,7 @@
       </c>
       <c r="C71" s="13" t="n">
         <f aca="false">'Targets 2027'!H10</f>
-        <v>269489.88</v>
+        <v>277064.62</v>
       </c>
       <c r="D71" s="16"/>
       <c r="E71" s="7" t="str">
@@ -3528,7 +3531,7 @@
       </c>
       <c r="C72" s="13" t="n">
         <f aca="false">'Targets 2027'!I10</f>
-        <v>274315.81</v>
+        <v>282316.14</v>
       </c>
       <c r="D72" s="16"/>
       <c r="E72" s="7" t="str">
@@ -3549,7 +3552,7 @@
       </c>
       <c r="C73" s="13" t="n">
         <f aca="false">'Targets 2027'!J10</f>
-        <v>238484.98</v>
+        <v>245303.53</v>
       </c>
       <c r="D73" s="16"/>
       <c r="E73" s="7" t="str">
@@ -3570,7 +3573,7 @@
       </c>
       <c r="C74" s="13" t="n">
         <f aca="false">'Targets 2027'!K10</f>
-        <v>252570.07</v>
+        <v>259853.16</v>
       </c>
       <c r="D74" s="16"/>
       <c r="E74" s="7" t="str">
@@ -3591,7 +3594,7 @@
       </c>
       <c r="C75" s="13" t="n">
         <f aca="false">'Targets 2027'!L10</f>
-        <v>244479.98</v>
+        <v>251500.08</v>
       </c>
       <c r="D75" s="16"/>
       <c r="E75" s="7" t="str">
@@ -3612,7 +3615,7 @@
       </c>
       <c r="C76" s="13" t="n">
         <f aca="false">'Targets 2027'!M10</f>
-        <v>256922.52</v>
+        <v>264190.98</v>
       </c>
       <c r="D76" s="16"/>
       <c r="E76" s="7" t="str">
@@ -3633,7 +3636,7 @@
       </c>
       <c r="C77" s="13" t="n">
         <f aca="false">'Targets 2027'!B11</f>
-        <v>68962.29</v>
+        <v>70800.15</v>
       </c>
       <c r="D77" s="16"/>
       <c r="E77" s="7" t="str">
@@ -3654,7 +3657,7 @@
       </c>
       <c r="C78" s="13" t="n">
         <f aca="false">'Targets 2027'!C11</f>
-        <v>64298.16</v>
+        <v>66007.9</v>
       </c>
       <c r="D78" s="16"/>
       <c r="E78" s="7" t="str">
@@ -3675,7 +3678,7 @@
       </c>
       <c r="C79" s="13" t="n">
         <f aca="false">'Targets 2027'!D11</f>
-        <v>80750.82</v>
+        <v>82990.05</v>
       </c>
       <c r="D79" s="16"/>
       <c r="E79" s="7" t="str">
@@ -3696,7 +3699,7 @@
       </c>
       <c r="C80" s="13" t="n">
         <f aca="false">'Targets 2027'!E11</f>
-        <v>76408.93</v>
+        <v>78388.91</v>
       </c>
       <c r="D80" s="16"/>
       <c r="E80" s="7" t="str">
@@ -3717,7 +3720,7 @@
       </c>
       <c r="C81" s="13" t="n">
         <f aca="false">'Targets 2027'!F11</f>
-        <v>81062.97</v>
+        <v>83243.53</v>
       </c>
       <c r="D81" s="16"/>
       <c r="E81" s="7" t="str">
@@ -3738,7 +3741,7 @@
       </c>
       <c r="C82" s="13" t="n">
         <f aca="false">'Targets 2027'!G11</f>
-        <v>79234.8</v>
+        <v>81334.93</v>
       </c>
       <c r="D82" s="16"/>
       <c r="E82" s="7" t="str">
@@ -3759,7 +3762,7 @@
       </c>
       <c r="C83" s="13" t="n">
         <f aca="false">'Targets 2027'!H11</f>
-        <v>93765.52</v>
+        <v>96269.06</v>
       </c>
       <c r="D83" s="16"/>
       <c r="E83" s="7" t="str">
@@ -3780,7 +3783,7 @@
       </c>
       <c r="C84" s="13" t="n">
         <f aca="false">'Targets 2027'!I11</f>
-        <v>92719.44</v>
+        <v>95278.83</v>
       </c>
       <c r="D84" s="16"/>
       <c r="E84" s="7" t="str">
@@ -3801,7 +3804,7 @@
       </c>
       <c r="C85" s="13" t="n">
         <f aca="false">'Targets 2027'!J11</f>
-        <v>73936.93</v>
+        <v>75882.64</v>
       </c>
       <c r="D85" s="16"/>
       <c r="E85" s="7" t="str">
@@ -3822,7 +3825,7 @@
       </c>
       <c r="C86" s="13" t="n">
         <f aca="false">'Targets 2027'!K11</f>
-        <v>72624.46</v>
+        <v>74528.35</v>
       </c>
       <c r="D86" s="16"/>
       <c r="E86" s="7" t="str">
@@ -3843,7 +3846,7 @@
       </c>
       <c r="C87" s="13" t="n">
         <f aca="false">'Targets 2027'!L11</f>
-        <v>66319.24</v>
+        <v>68063.03</v>
       </c>
       <c r="D87" s="16"/>
       <c r="E87" s="7" t="str">
@@ -3864,7 +3867,7 @@
       </c>
       <c r="C88" s="13" t="n">
         <f aca="false">'Targets 2027'!M11</f>
-        <v>67419.34</v>
+        <v>69162.45</v>
       </c>
       <c r="D88" s="16"/>
       <c r="E88" s="7" t="str">
@@ -4137,7 +4140,7 @@
       </c>
       <c r="C101" s="13" t="n">
         <f aca="false">'Targets 2027'!B13</f>
-        <v>310339.79</v>
+        <v>313961.18</v>
       </c>
       <c r="D101" s="16"/>
       <c r="E101" s="7" t="str">
@@ -4158,7 +4161,7 @@
       </c>
       <c r="C102" s="13" t="n">
         <f aca="false">'Targets 2027'!C13</f>
-        <v>261447.34</v>
+        <v>264597.31</v>
       </c>
       <c r="D102" s="16"/>
       <c r="E102" s="7" t="str">
@@ -4179,7 +4182,7 @@
       </c>
       <c r="C103" s="13" t="n">
         <f aca="false">'Targets 2027'!D13</f>
-        <v>310773.11</v>
+        <v>314664.44</v>
       </c>
       <c r="D103" s="16"/>
       <c r="E103" s="7" t="str">
@@ -4200,7 +4203,7 @@
       </c>
       <c r="C104" s="13" t="n">
         <f aca="false">'Targets 2027'!E13</f>
-        <v>296667.43</v>
+        <v>300264.21</v>
       </c>
       <c r="D104" s="16"/>
       <c r="E104" s="7" t="str">
@@ -4221,7 +4224,7 @@
       </c>
       <c r="C105" s="13" t="n">
         <f aca="false">'Targets 2027'!F13</f>
-        <v>339151.24</v>
+        <v>343298.88</v>
       </c>
       <c r="D105" s="16"/>
       <c r="E105" s="7" t="str">
@@ -4242,7 +4245,7 @@
       </c>
       <c r="C106" s="13" t="n">
         <f aca="false">'Targets 2027'!G13</f>
-        <v>316744.84</v>
+        <v>320623.44</v>
       </c>
       <c r="D106" s="16"/>
       <c r="E106" s="7" t="str">
@@ -4263,7 +4266,7 @@
       </c>
       <c r="C107" s="13" t="n">
         <f aca="false">'Targets 2027'!H13</f>
-        <v>349578</v>
+        <v>353788.55</v>
       </c>
       <c r="D107" s="16"/>
       <c r="E107" s="7" t="str">
@@ -4284,7 +4287,7 @@
       </c>
       <c r="C108" s="13" t="n">
         <f aca="false">'Targets 2027'!I13</f>
-        <v>352910.43</v>
+        <v>357326.1</v>
       </c>
       <c r="D108" s="16"/>
       <c r="E108" s="7" t="str">
@@ -4305,7 +4308,7 @@
       </c>
       <c r="C109" s="13" t="n">
         <f aca="false">'Targets 2027'!J13</f>
-        <v>285576.59</v>
+        <v>289029.4</v>
       </c>
       <c r="D109" s="16"/>
       <c r="E109" s="7" t="str">
@@ -4326,7 +4329,7 @@
       </c>
       <c r="C110" s="13" t="n">
         <f aca="false">'Targets 2027'!K13</f>
-        <v>300807.14</v>
+        <v>304308.3</v>
       </c>
       <c r="D110" s="16"/>
       <c r="E110" s="7" t="str">
@@ -4347,7 +4350,7 @@
       </c>
       <c r="C111" s="13" t="n">
         <f aca="false">'Targets 2027'!L13</f>
-        <v>287803.85</v>
+        <v>291298.45</v>
       </c>
       <c r="D111" s="16"/>
       <c r="E111" s="7" t="str">
@@ -4368,7 +4371,7 @@
       </c>
       <c r="C112" s="13" t="n">
         <f aca="false">'Targets 2027'!M13</f>
-        <v>306150.86</v>
+        <v>309737.62</v>
       </c>
       <c r="D112" s="16"/>
       <c r="E112" s="7" t="str">
@@ -4648,7 +4651,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -4712,11 +4715,11 @@
       </c>
       <c r="G5" s="13" t="n">
         <f aca="false">'Targets 2027'!R5</f>
-        <v>2939876.01</v>
+        <v>3027430.33</v>
       </c>
       <c r="H5" s="7" t="n">
         <f aca="false">G5-E5</f>
-        <v>182120.2</v>
+        <v>269674.52</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4792,15 +4795,15 @@
         <v>4134497.38</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>3929309.57</v>
+        <v>4035313.38</v>
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">'Targets 2027'!R8</f>
-        <v>4195611.3</v>
+        <v>4301615.09</v>
       </c>
       <c r="H8" s="7" t="n">
         <f aca="false">G8-E8</f>
-        <v>61113.9199999999</v>
+        <v>167117.71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4852,11 +4855,11 @@
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">'Targets 2027'!R10</f>
-        <v>3049343.66</v>
+        <v>3136466.32</v>
       </c>
       <c r="H10" s="7" t="n">
         <f aca="false">G10-E10</f>
-        <v>7590.45999999996</v>
+        <v>94713.1199999997</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4876,15 +4879,15 @@
         <v>936771.96</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>880008.54</v>
+        <v>904455.5</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">'Targets 2027'!R11</f>
-        <v>917502.9</v>
+        <v>941949.83</v>
       </c>
       <c r="H11" s="7" t="n">
         <f aca="false">G11-E11</f>
-        <v>-19269.0599999999</v>
+        <v>5177.87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4932,15 +4935,15 @@
         <v>3606994.37</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>3485293.26</v>
+        <v>3530240.52</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">'Targets 2027'!R13</f>
-        <v>3717950.62</v>
+        <v>3762897.88</v>
       </c>
       <c r="H13" s="7" t="n">
         <f aca="false">G13-E13</f>
-        <v>110956.25</v>
+        <v>155903.51</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4993,20 +4996,25 @@
       </c>
       <c r="F15" s="10" t="n">
         <f aca="false">SUM(F5:F14)</f>
-        <v>29580590.48</v>
+        <v>29755988.51</v>
       </c>
       <c r="G15" s="10" t="n">
         <f aca="false">SUM(G5:G14)</f>
-        <v>30956827.3</v>
+        <v>31306902.26</v>
       </c>
       <c r="H15" s="10" t="n">
         <f aca="false">SUM(H5:H14)</f>
-        <v>1271196.33</v>
+        <v>1621271.29</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>